<commit_message>
feat(reports): complete weekly charts and clarify matched data costs
</commit_message>
<xml_diff>
--- a/tuan_1/docs/Bao_cao_tuan_1_Du_lieu_Athena_24110054_24110051.xlsx
+++ b/tuan_1/docs/Bao_cao_tuan_1_Du_lieu_Athena_24110054_24110051.xlsx
@@ -7,6 +7,7 @@
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phân bố AQI" sheetId="3" r:id="Rd93c90fe9a9a4a8c"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tương quan" sheetId="4" r:id="R49fe31345d3c4d54"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="156 bản ghi gốc" sheetId="5" r:id="Rb9117e2fe3b4443c"/>
+    <x:sheet xmlns:ns0="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phan_tich_bo_sung" sheetId="6" ns0:id="rId1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,15 +18,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="8">
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
     <x:numFmt numFmtId="201" formatCode="0.00"/>
     <x:numFmt numFmtId="202" formatCode="00"/>
     <x:numFmt numFmtId="203" formatCode="0.0&quot;%&quot;"/>
     <x:numFmt numFmtId="204" formatCode="0.0000"/>
     <x:numFmt numFmtId="205" formatCode="yyyy-mm-dd&quot;T&quot;hh:mm:ss&quot;+00:00&quot;"/>
+    <x:numFmt numFmtId="206" formatCode="0.00"/>
+    <x:numFmt numFmtId="207" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -47,8 +50,29 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Times New Roman"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Times New Roman"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Times New Roman"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -65,8 +89,19 @@
         <x:fgColor rgb="FFF2F2F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="none"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7E7E7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="4">
+  <x:borders count="5">
     <x:border>
       <x:left/>
       <x:right/>
@@ -103,11 +138,19 @@
       <x:bottom/>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
-  <x:cellStyleXfs count="1">
+  <x:cellStyleXfs count="2">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="62">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -248,6 +291,36 @@
     <x:xf numFmtId="200" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="6" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="7" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="7" fillId="6" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="7" fillId="6" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="7" fillId="6" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="6" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="6" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="6" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -370,6 +443,146 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc0df5b5322c64a56"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="9144000" cy="4953000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="d04cb0cf-a995-4244-a52e-0a395b5bd89a"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R700fce09373641c7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="9144000" cy="4953000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="777dba0c-36c6-40b5-9d02-5d708b631c07"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7248888453834710"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="9144000" cy="4953000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="e7b1b649-adb0-4d4c-a94a-0101ab56aae5"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rfe7141243c924ac7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>87</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="9144000" cy="4953000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="d9e60086-2e4f-4b3d-a3ec-9b1779145c2e"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R92af5d07f9954456"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>115</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="9144000" cy="4953000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="f200cc18-070e-4212-b63e-4a16c4f9dd85"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R361a74e72ca64bda"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -12698,4 +12911,984 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="36" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="17" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="17" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="51" t="str">
+        <x:v>Phân tích bổ sung dữ liệu Tuần 1</x:v>
+      </x:c>
+      <x:c r="B2" s="51"/>
+      <x:c r="C2" s="51"/>
+      <x:c r="D2" s="51"/>
+      <x:c r="E2" s="51"/>
+      <x:c r="F2" s="51"/>
+      <x:c r="G2" s="51"/>
+      <x:c r="H2" s="51"/>
+      <x:c r="I2" s="51"/>
+      <x:c r="J2" s="51"/>
+      <x:c r="K2" s="51"/>
+      <x:c r="L2" s="51"/>
+    </x:row>
+    <x:row r="4" ht="34" customHeight="1">
+      <x:c r="A4" s="58" t="str">
+        <x:v>city</x:v>
+      </x:c>
+      <x:c r="B4" s="58" t="str">
+        <x:v>city_label</x:v>
+      </x:c>
+      <x:c r="C4" s="58" t="str">
+        <x:v>variable</x:v>
+      </x:c>
+      <x:c r="D4" s="58" t="str">
+        <x:v>unit</x:v>
+      </x:c>
+      <x:c r="E4" s="58" t="str">
+        <x:v>n</x:v>
+      </x:c>
+      <x:c r="F4" s="58" t="str">
+        <x:v>mean</x:v>
+      </x:c>
+      <x:c r="G4" s="58" t="str">
+        <x:v>sd</x:v>
+      </x:c>
+      <x:c r="H4" s="58" t="str">
+        <x:v>min</x:v>
+      </x:c>
+      <x:c r="I4" s="58" t="str">
+        <x:v>q1</x:v>
+      </x:c>
+      <x:c r="J4" s="58" t="str">
+        <x:v>median</x:v>
+      </x:c>
+      <x:c r="K4" s="58" t="str">
+        <x:v>q3</x:v>
+      </x:c>
+      <x:c r="L4" s="58" t="str">
+        <x:v>p95</x:v>
+      </x:c>
+      <x:c r="M4" s="58" t="str">
+        <x:v>max</x:v>
+      </x:c>
+      <x:c r="N4" s="58" t="str">
+        <x:v>pearson_pm25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="59" t="str">
+        <x:v>HoChiMinh</x:v>
+      </x:c>
+      <x:c r="B5" s="59" t="str">
+        <x:v>TP. Hồ Chí Minh</x:v>
+      </x:c>
+      <x:c r="C5" s="59" t="str">
+        <x:v>us_aqi</x:v>
+      </x:c>
+      <x:c r="D5" s="59" t="str">
+        <x:v>US AQI</x:v>
+      </x:c>
+      <x:c r="E5" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F5" s="60" t="n">
+        <x:v>107.78846153846153</x:v>
+      </x:c>
+      <x:c r="G5" s="60" t="n">
+        <x:v>17.84940987486266</x:v>
+      </x:c>
+      <x:c r="H5" s="60" t="n">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="I5" s="60" t="n">
+        <x:v>100.75</x:v>
+      </x:c>
+      <x:c r="J5" s="60" t="n">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="K5" s="60" t="n">
+        <x:v>106.5</x:v>
+      </x:c>
+      <x:c r="L5" s="60" t="n">
+        <x:v>156.49999999999994</x:v>
+      </x:c>
+      <x:c r="M5" s="60" t="n">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="N5" s="60" t="n">
+        <x:v>0.03507836922700715</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="59" t="str">
+        <x:v>HoChiMinh</x:v>
+      </x:c>
+      <x:c r="B6" s="59" t="str">
+        <x:v>TP. Hồ Chí Minh</x:v>
+      </x:c>
+      <x:c r="C6" s="59" t="str">
+        <x:v>pm2_5</x:v>
+      </x:c>
+      <x:c r="D6" s="59" t="str">
+        <x:v>µg/m³</x:v>
+      </x:c>
+      <x:c r="E6" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F6" s="60" t="n">
+        <x:v>37.03076923076923</x:v>
+      </x:c>
+      <x:c r="G6" s="60" t="n">
+        <x:v>9.546327462649325</x:v>
+      </x:c>
+      <x:c r="H6" s="60" t="n">
+        <x:v>20.2</x:v>
+      </x:c>
+      <x:c r="I6" s="60" t="n">
+        <x:v>30.849999999999998</x:v>
+      </x:c>
+      <x:c r="J6" s="60" t="n">
+        <x:v>36.5</x:v>
+      </x:c>
+      <x:c r="K6" s="60" t="n">
+        <x:v>39.9</x:v>
+      </x:c>
+      <x:c r="L6" s="60" t="n">
+        <x:v>55.66</x:v>
+      </x:c>
+      <x:c r="M6" s="60" t="n">
+        <x:v>59.8</x:v>
+      </x:c>
+      <x:c r="N6" s="60" t="n">
+        <x:v>0.9999999999999998</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="59" t="str">
+        <x:v>HoChiMinh</x:v>
+      </x:c>
+      <x:c r="B7" s="59" t="str">
+        <x:v>TP. Hồ Chí Minh</x:v>
+      </x:c>
+      <x:c r="C7" s="59" t="str">
+        <x:v>pm10</x:v>
+      </x:c>
+      <x:c r="D7" s="59" t="str">
+        <x:v>µg/m³</x:v>
+      </x:c>
+      <x:c r="E7" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F7" s="60" t="n">
+        <x:v>37.35192307692308</x:v>
+      </x:c>
+      <x:c r="G7" s="60" t="n">
+        <x:v>9.417224319103784</x:v>
+      </x:c>
+      <x:c r="H7" s="60" t="n">
+        <x:v>20.4</x:v>
+      </x:c>
+      <x:c r="I7" s="60" t="n">
+        <x:v>31.275</x:v>
+      </x:c>
+      <x:c r="J7" s="60" t="n">
+        <x:v>36.7</x:v>
+      </x:c>
+      <x:c r="K7" s="60" t="n">
+        <x:v>40.1</x:v>
+      </x:c>
+      <x:c r="L7" s="60" t="n">
+        <x:v>55.76</x:v>
+      </x:c>
+      <x:c r="M7" s="60" t="n">
+        <x:v>59.8</x:v>
+      </x:c>
+      <x:c r="N7" s="60" t="n">
+        <x:v>0.9993045989388457</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="59" t="str">
+        <x:v>HoChiMinh</x:v>
+      </x:c>
+      <x:c r="B8" s="59" t="str">
+        <x:v>TP. Hồ Chí Minh</x:v>
+      </x:c>
+      <x:c r="C8" s="59" t="str">
+        <x:v>temperature_2m</x:v>
+      </x:c>
+      <x:c r="D8" s="59" t="str">
+        <x:v>°C</x:v>
+      </x:c>
+      <x:c r="E8" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F8" s="60" t="n">
+        <x:v>27.788461538461544</x:v>
+      </x:c>
+      <x:c r="G8" s="60" t="n">
+        <x:v>2.3142909680431742</x:v>
+      </x:c>
+      <x:c r="H8" s="60" t="n">
+        <x:v>24.3</x:v>
+      </x:c>
+      <x:c r="I8" s="60" t="n">
+        <x:v>26.25</x:v>
+      </x:c>
+      <x:c r="J8" s="60" t="n">
+        <x:v>27.2</x:v>
+      </x:c>
+      <x:c r="K8" s="60" t="n">
+        <x:v>29.3</x:v>
+      </x:c>
+      <x:c r="L8" s="60" t="n">
+        <x:v>32.235</x:v>
+      </x:c>
+      <x:c r="M8" s="60" t="n">
+        <x:v>33.3</x:v>
+      </x:c>
+      <x:c r="N8" s="60" t="n">
+        <x:v>-0.6977387661815306</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="59" t="str">
+        <x:v>HoChiMinh</x:v>
+      </x:c>
+      <x:c r="B9" s="59" t="str">
+        <x:v>TP. Hồ Chí Minh</x:v>
+      </x:c>
+      <x:c r="C9" s="59" t="str">
+        <x:v>relative_humidity_2m</x:v>
+      </x:c>
+      <x:c r="D9" s="59" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="E9" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F9" s="60" t="n">
+        <x:v>84.71153846153847</x:v>
+      </x:c>
+      <x:c r="G9" s="60" t="n">
+        <x:v>12.451217026052685</x:v>
+      </x:c>
+      <x:c r="H9" s="60" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="I9" s="60" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="J9" s="60" t="n">
+        <x:v>88.5</x:v>
+      </x:c>
+      <x:c r="K9" s="60" t="n">
+        <x:v>95.25</x:v>
+      </x:c>
+      <x:c r="L9" s="60" t="n">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="M9" s="60" t="n">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="N9" s="60" t="n">
+        <x:v>0.6627086063443471</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="59" t="str">
+        <x:v>HoChiMinh</x:v>
+      </x:c>
+      <x:c r="B10" s="59" t="str">
+        <x:v>TP. Hồ Chí Minh</x:v>
+      </x:c>
+      <x:c r="C10" s="59" t="str">
+        <x:v>wind_speed_10m</x:v>
+      </x:c>
+      <x:c r="D10" s="59" t="str">
+        <x:v>km/h</x:v>
+      </x:c>
+      <x:c r="E10" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F10" s="60" t="n">
+        <x:v>4.121153846153846</x:v>
+      </x:c>
+      <x:c r="G10" s="60" t="n">
+        <x:v>2.438123397483701</x:v>
+      </x:c>
+      <x:c r="H10" s="60" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="I10" s="60" t="n">
+        <x:v>2.375</x:v>
+      </x:c>
+      <x:c r="J10" s="60" t="n">
+        <x:v>3.8</x:v>
+      </x:c>
+      <x:c r="K10" s="60" t="n">
+        <x:v>5.5</x:v>
+      </x:c>
+      <x:c r="L10" s="60" t="n">
+        <x:v>7.769999999999997</x:v>
+      </x:c>
+      <x:c r="M10" s="60" t="n">
+        <x:v>13.2</x:v>
+      </x:c>
+      <x:c r="N10" s="60" t="n">
+        <x:v>-0.1535964887795929</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="59" t="str">
+        <x:v>HaNoi</x:v>
+      </x:c>
+      <x:c r="B11" s="59" t="str">
+        <x:v>Hà Nội</x:v>
+      </x:c>
+      <x:c r="C11" s="59" t="str">
+        <x:v>us_aqi</x:v>
+      </x:c>
+      <x:c r="D11" s="59" t="str">
+        <x:v>US AQI</x:v>
+      </x:c>
+      <x:c r="E11" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F11" s="60" t="n">
+        <x:v>67.5576923076923</x:v>
+      </x:c>
+      <x:c r="G11" s="60" t="n">
+        <x:v>9.945761658228724</x:v>
+      </x:c>
+      <x:c r="H11" s="60" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="I11" s="60" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="J11" s="60" t="n">
+        <x:v>65.5</x:v>
+      </x:c>
+      <x:c r="K11" s="60" t="n">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="L11" s="60" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="M11" s="60" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="N11" s="60" t="n">
+        <x:v>0.46264519840443225</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="59" t="str">
+        <x:v>HaNoi</x:v>
+      </x:c>
+      <x:c r="B12" s="59" t="str">
+        <x:v>Hà Nội</x:v>
+      </x:c>
+      <x:c r="C12" s="59" t="str">
+        <x:v>pm2_5</x:v>
+      </x:c>
+      <x:c r="D12" s="59" t="str">
+        <x:v>µg/m³</x:v>
+      </x:c>
+      <x:c r="E12" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F12" s="60" t="n">
+        <x:v>15.363461538461538</x:v>
+      </x:c>
+      <x:c r="G12" s="60" t="n">
+        <x:v>5.892801485832768</x:v>
+      </x:c>
+      <x:c r="H12" s="60" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="I12" s="60" t="n">
+        <x:v>10.95</x:v>
+      </x:c>
+      <x:c r="J12" s="60" t="n">
+        <x:v>12.850000000000001</x:v>
+      </x:c>
+      <x:c r="K12" s="60" t="n">
+        <x:v>20.95</x:v>
+      </x:c>
+      <x:c r="L12" s="60" t="n">
+        <x:v>26.019999999999992</x:v>
+      </x:c>
+      <x:c r="M12" s="60" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="N12" s="60" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="59" t="str">
+        <x:v>HaNoi</x:v>
+      </x:c>
+      <x:c r="B13" s="59" t="str">
+        <x:v>Hà Nội</x:v>
+      </x:c>
+      <x:c r="C13" s="59" t="str">
+        <x:v>pm10</x:v>
+      </x:c>
+      <x:c r="D13" s="59" t="str">
+        <x:v>µg/m³</x:v>
+      </x:c>
+      <x:c r="E13" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F13" s="60" t="n">
+        <x:v>16.109615384615385</x:v>
+      </x:c>
+      <x:c r="G13" s="60" t="n">
+        <x:v>6.435144303130398</x:v>
+      </x:c>
+      <x:c r="H13" s="60" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="I13" s="60" t="n">
+        <x:v>11.075</x:v>
+      </x:c>
+      <x:c r="J13" s="60" t="n">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="K13" s="60" t="n">
+        <x:v>22.325</x:v>
+      </x:c>
+      <x:c r="L13" s="60" t="n">
+        <x:v>27.979999999999997</x:v>
+      </x:c>
+      <x:c r="M13" s="60" t="n">
+        <x:v>29.6</x:v>
+      </x:c>
+      <x:c r="N13" s="60" t="n">
+        <x:v>0.9888963493111396</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="59" t="str">
+        <x:v>HaNoi</x:v>
+      </x:c>
+      <x:c r="B14" s="59" t="str">
+        <x:v>Hà Nội</x:v>
+      </x:c>
+      <x:c r="C14" s="59" t="str">
+        <x:v>temperature_2m</x:v>
+      </x:c>
+      <x:c r="D14" s="59" t="str">
+        <x:v>°C</x:v>
+      </x:c>
+      <x:c r="E14" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F14" s="60" t="n">
+        <x:v>24.536538461538463</x:v>
+      </x:c>
+      <x:c r="G14" s="60" t="n">
+        <x:v>1.8900180356182565</x:v>
+      </x:c>
+      <x:c r="H14" s="60" t="n">
+        <x:v>21.9</x:v>
+      </x:c>
+      <x:c r="I14" s="60" t="n">
+        <x:v>23.075000000000003</x:v>
+      </x:c>
+      <x:c r="J14" s="60" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="K14" s="60" t="n">
+        <x:v>25.8</x:v>
+      </x:c>
+      <x:c r="L14" s="60" t="n">
+        <x:v>27.834999999999997</x:v>
+      </x:c>
+      <x:c r="M14" s="60" t="n">
+        <x:v>29.3</x:v>
+      </x:c>
+      <x:c r="N14" s="60" t="n">
+        <x:v>0.646181883679886</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="59" t="str">
+        <x:v>HaNoi</x:v>
+      </x:c>
+      <x:c r="B15" s="59" t="str">
+        <x:v>Hà Nội</x:v>
+      </x:c>
+      <x:c r="C15" s="59" t="str">
+        <x:v>relative_humidity_2m</x:v>
+      </x:c>
+      <x:c r="D15" s="59" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="E15" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F15" s="60" t="n">
+        <x:v>76.65384615384616</x:v>
+      </x:c>
+      <x:c r="G15" s="60" t="n">
+        <x:v>13.207075666556234</x:v>
+      </x:c>
+      <x:c r="H15" s="60" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="I15" s="60" t="n">
+        <x:v>64.75</x:v>
+      </x:c>
+      <x:c r="J15" s="60" t="n">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="K15" s="60" t="n">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="L15" s="60" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="M15" s="60" t="n">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="N15" s="60" t="n">
+        <x:v>0.2486022736861401</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="59" t="str">
+        <x:v>HaNoi</x:v>
+      </x:c>
+      <x:c r="B16" s="59" t="str">
+        <x:v>Hà Nội</x:v>
+      </x:c>
+      <x:c r="C16" s="59" t="str">
+        <x:v>wind_speed_10m</x:v>
+      </x:c>
+      <x:c r="D16" s="59" t="str">
+        <x:v>km/h</x:v>
+      </x:c>
+      <x:c r="E16" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F16" s="60" t="n">
+        <x:v>12.084615384615386</x:v>
+      </x:c>
+      <x:c r="G16" s="60" t="n">
+        <x:v>3.3420895550940095</x:v>
+      </x:c>
+      <x:c r="H16" s="60" t="n">
+        <x:v>5.2</x:v>
+      </x:c>
+      <x:c r="I16" s="60" t="n">
+        <x:v>9.95</x:v>
+      </x:c>
+      <x:c r="J16" s="60" t="n">
+        <x:v>12.45</x:v>
+      </x:c>
+      <x:c r="K16" s="60" t="n">
+        <x:v>14.55</x:v>
+      </x:c>
+      <x:c r="L16" s="60" t="n">
+        <x:v>16.825</x:v>
+      </x:c>
+      <x:c r="M16" s="60" t="n">
+        <x:v>17.9</x:v>
+      </x:c>
+      <x:c r="N16" s="60" t="n">
+        <x:v>-0.48462311621929105</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="59" t="str">
+        <x:v>DaNang</x:v>
+      </x:c>
+      <x:c r="B17" s="59" t="str">
+        <x:v>Đà Nẵng</x:v>
+      </x:c>
+      <x:c r="C17" s="59" t="str">
+        <x:v>us_aqi</x:v>
+      </x:c>
+      <x:c r="D17" s="59" t="str">
+        <x:v>US AQI</x:v>
+      </x:c>
+      <x:c r="E17" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F17" s="60" t="n">
+        <x:v>74.67307692307692</x:v>
+      </x:c>
+      <x:c r="G17" s="60" t="n">
+        <x:v>28.846939657471637</x:v>
+      </x:c>
+      <x:c r="H17" s="60" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="I17" s="60" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="J17" s="60" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="K17" s="60" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="L17" s="60" t="n">
+        <x:v>143.84999999999994</x:v>
+      </x:c>
+      <x:c r="M17" s="60" t="n">
+        <x:v>155</x:v>
+      </x:c>
+      <x:c r="N17" s="60" t="n">
+        <x:v>0.38036982665471114</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="59" t="str">
+        <x:v>DaNang</x:v>
+      </x:c>
+      <x:c r="B18" s="59" t="str">
+        <x:v>Đà Nẵng</x:v>
+      </x:c>
+      <x:c r="C18" s="59" t="str">
+        <x:v>pm2_5</x:v>
+      </x:c>
+      <x:c r="D18" s="59" t="str">
+        <x:v>µg/m³</x:v>
+      </x:c>
+      <x:c r="E18" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F18" s="60" t="n">
+        <x:v>14.232692307692306</x:v>
+      </x:c>
+      <x:c r="G18" s="60" t="n">
+        <x:v>9.932590862247494</x:v>
+      </x:c>
+      <x:c r="H18" s="60" t="n">
+        <x:v>2.6</x:v>
+      </x:c>
+      <x:c r="I18" s="60" t="n">
+        <x:v>6.4</x:v>
+      </x:c>
+      <x:c r="J18" s="60" t="n">
+        <x:v>8.8</x:v>
+      </x:c>
+      <x:c r="K18" s="60" t="n">
+        <x:v>24.95</x:v>
+      </x:c>
+      <x:c r="L18" s="60" t="n">
+        <x:v>30.394999999999996</x:v>
+      </x:c>
+      <x:c r="M18" s="60" t="n">
+        <x:v>33.2</x:v>
+      </x:c>
+      <x:c r="N18" s="60" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="24" customHeight="1">
+      <x:c r="A19" s="59" t="str">
+        <x:v>DaNang</x:v>
+      </x:c>
+      <x:c r="B19" s="59" t="str">
+        <x:v>Đà Nẵng</x:v>
+      </x:c>
+      <x:c r="C19" s="59" t="str">
+        <x:v>pm10</x:v>
+      </x:c>
+      <x:c r="D19" s="59" t="str">
+        <x:v>µg/m³</x:v>
+      </x:c>
+      <x:c r="E19" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F19" s="60" t="n">
+        <x:v>17.276923076923076</x:v>
+      </x:c>
+      <x:c r="G19" s="60" t="n">
+        <x:v>10.91826344348852</x:v>
+      </x:c>
+      <x:c r="H19" s="60" t="n">
+        <x:v>3.1</x:v>
+      </x:c>
+      <x:c r="I19" s="60" t="n">
+        <x:v>8.725000000000001</x:v>
+      </x:c>
+      <x:c r="J19" s="60" t="n">
+        <x:v>12.3</x:v>
+      </x:c>
+      <x:c r="K19" s="60" t="n">
+        <x:v>28.925</x:v>
+      </x:c>
+      <x:c r="L19" s="60" t="n">
+        <x:v>33.48499999999999</x:v>
+      </x:c>
+      <x:c r="M19" s="60" t="n">
+        <x:v>37.8</x:v>
+      </x:c>
+      <x:c r="N19" s="60" t="n">
+        <x:v>0.9965972968649626</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="24" customHeight="1">
+      <x:c r="A20" s="59" t="str">
+        <x:v>DaNang</x:v>
+      </x:c>
+      <x:c r="B20" s="59" t="str">
+        <x:v>Đà Nẵng</x:v>
+      </x:c>
+      <x:c r="C20" s="59" t="str">
+        <x:v>temperature_2m</x:v>
+      </x:c>
+      <x:c r="D20" s="59" t="str">
+        <x:v>°C</x:v>
+      </x:c>
+      <x:c r="E20" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F20" s="60" t="n">
+        <x:v>28.84615384615385</x:v>
+      </x:c>
+      <x:c r="G20" s="60" t="n">
+        <x:v>2.9088412583128958</x:v>
+      </x:c>
+      <x:c r="H20" s="60" t="n">
+        <x:v>23.9</x:v>
+      </x:c>
+      <x:c r="I20" s="60" t="n">
+        <x:v>26.45</x:v>
+      </x:c>
+      <x:c r="J20" s="60" t="n">
+        <x:v>28.9</x:v>
+      </x:c>
+      <x:c r="K20" s="60" t="n">
+        <x:v>31.175</x:v>
+      </x:c>
+      <x:c r="L20" s="60" t="n">
+        <x:v>33.045</x:v>
+      </x:c>
+      <x:c r="M20" s="60" t="n">
+        <x:v>33.4</x:v>
+      </x:c>
+      <x:c r="N20" s="60" t="n">
+        <x:v>0.4797674242404333</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="24" customHeight="1">
+      <x:c r="A21" s="59" t="str">
+        <x:v>DaNang</x:v>
+      </x:c>
+      <x:c r="B21" s="59" t="str">
+        <x:v>Đà Nẵng</x:v>
+      </x:c>
+      <x:c r="C21" s="59" t="str">
+        <x:v>relative_humidity_2m</x:v>
+      </x:c>
+      <x:c r="D21" s="59" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="E21" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F21" s="60" t="n">
+        <x:v>74.86538461538461</x:v>
+      </x:c>
+      <x:c r="G21" s="60" t="n">
+        <x:v>14.44398082947051</x:v>
+      </x:c>
+      <x:c r="H21" s="60" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="I21" s="60" t="n">
+        <x:v>60.75</x:v>
+      </x:c>
+      <x:c r="J21" s="60" t="n">
+        <x:v>76.5</x:v>
+      </x:c>
+      <x:c r="K21" s="60" t="n">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="L21" s="60" t="n">
+        <x:v>94.44999999999999</x:v>
+      </x:c>
+      <x:c r="M21" s="60" t="n">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="N21" s="60" t="n">
+        <x:v>-0.3182920823797298</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="24" customHeight="1">
+      <x:c r="A22" s="59" t="str">
+        <x:v>DaNang</x:v>
+      </x:c>
+      <x:c r="B22" s="59" t="str">
+        <x:v>Đà Nẵng</x:v>
+      </x:c>
+      <x:c r="C22" s="59" t="str">
+        <x:v>wind_speed_10m</x:v>
+      </x:c>
+      <x:c r="D22" s="59" t="str">
+        <x:v>km/h</x:v>
+      </x:c>
+      <x:c r="E22" s="61" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F22" s="60" t="n">
+        <x:v>8.411538461538463</x:v>
+      </x:c>
+      <x:c r="G22" s="60" t="n">
+        <x:v>4.7072182304499055</x:v>
+      </x:c>
+      <x:c r="H22" s="60" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="I22" s="60" t="n">
+        <x:v>5.3500000000000005</x:v>
+      </x:c>
+      <x:c r="J22" s="60" t="n">
+        <x:v>7.699999999999999</x:v>
+      </x:c>
+      <x:c r="K22" s="60" t="n">
+        <x:v>11.325000000000001</x:v>
+      </x:c>
+      <x:c r="L22" s="60" t="n">
+        <x:v>17.89</x:v>
+      </x:c>
+      <x:c r="M22" s="60" t="n">
+        <x:v>20.1</x:v>
+      </x:c>
+      <x:c r="N22" s="60" t="n">
+        <x:v>-0.2291046157747858</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="34" customHeight="1">
+      <x:c r="A27" s="58" t="str">
+        <x:v>Truy vấn</x:v>
+      </x:c>
+      <x:c r="B27" s="58" t="str">
+        <x:v>Trạng thái</x:v>
+      </x:c>
+      <x:c r="C27" s="58" t="str">
+        <x:v>Dòng kết quả</x:v>
+      </x:c>
+      <x:c r="D27" s="58" t="str">
+        <x:v>Thời gian ms</x:v>
+      </x:c>
+      <x:c r="E27" s="58" t="str">
+        <x:v>Byte quét</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="24" customHeight="1">
+      <x:c r="A28" s="59" t="str">
+        <x:v>avg_aqi_by_city</x:v>
+      </x:c>
+      <x:c r="B28" s="59" t="str">
+        <x:v>SUCCEEDED</x:v>
+      </x:c>
+      <x:c r="C28" s="61" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D28" s="61" t="n">
+        <x:v>744</x:v>
+      </x:c>
+      <x:c r="E28" s="61" t="n">
+        <x:v>87250</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="24" customHeight="1">
+      <x:c r="A29" s="59" t="str">
+        <x:v>peak_pollution_hours</x:v>
+      </x:c>
+      <x:c r="B29" s="59" t="str">
+        <x:v>SUCCEEDED</x:v>
+      </x:c>
+      <x:c r="C29" s="61" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="D29" s="61" t="n">
+        <x:v>936</x:v>
+      </x:c>
+      <x:c r="E29" s="61" t="n">
+        <x:v>87250</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="24" customHeight="1">
+      <x:c r="A30" s="59" t="str">
+        <x:v>aqi_category_distribution</x:v>
+      </x:c>
+      <x:c r="B30" s="59" t="str">
+        <x:v>SUCCEEDED</x:v>
+      </x:c>
+      <x:c r="C30" s="61" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D30" s="61" t="n">
+        <x:v>776</x:v>
+      </x:c>
+      <x:c r="E30" s="61" t="n">
+        <x:v>87250</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="24" customHeight="1">
+      <x:c r="A31" s="59" t="str">
+        <x:v>weather_correlation</x:v>
+      </x:c>
+      <x:c r="B31" s="59" t="str">
+        <x:v>SUCCEEDED</x:v>
+      </x:c>
+      <x:c r="C31" s="61" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D31" s="61" t="n">
+        <x:v>930</x:v>
+      </x:c>
+      <x:c r="E31" s="61" t="n">
+        <x:v>87250</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="24" customHeight="1">
+      <x:c r="A32" s="59" t="str">
+        <x:v>raw_weather_aqi_records</x:v>
+      </x:c>
+      <x:c r="B32" s="59" t="str">
+        <x:v>SUCCEEDED</x:v>
+      </x:c>
+      <x:c r="C32" s="61" t="n">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="D32" s="61" t="n">
+        <x:v>1192</x:v>
+      </x:c>
+      <x:c r="E32" s="61" t="n">
+        <x:v>87250</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b5cd57879c44bc0"/>
+</x:worksheet>
 </file>
</xml_diff>